<commit_message>
Ajustando exportacion de programas de maquinaria
</commit_message>
<xml_diff>
--- a/public/plantillas/11_PROG_UTILIZACION_EQUIPO.xlsx
+++ b/public/plantillas/11_PROG_UTILIZACION_EQUIPO.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E857B36C-0084-BE41-A4A0-C7AB05D3EE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB48002-6F1D-744F-BE83-C553D11B7AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3620" yWindow="0" windowWidth="29980" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MANTENIMIENTO FEBRERO 2024" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$A$1:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -734,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U985"/>
+  <dimension ref="A1:U984"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
@@ -822,67 +822,58 @@
       <c r="G5" s="7"/>
       <c r="H5" s="6"/>
     </row>
-    <row r="6" spans="1:21" ht="157" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="1:21" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="23" t="s">
+    <row r="6" spans="1:21" ht="69" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="14"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="14"/>
     </row>
-    <row r="8" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="17" t="s">
+    <row r="7" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="18" t="s">
+      <c r="D7" s="16"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
     </row>
-    <row r="9" spans="1:21" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
+    <row r="8" spans="1:21" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="19"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
     </row>
-    <row r="10" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="11" spans="1:21" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="12" spans="1:21" ht="8.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="9" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="10" spans="1:21" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:21" ht="8.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="12" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="13" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="14" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="15" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -1855,7 +1846,6 @@
     <row r="982" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="983" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="984" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="985" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:H1"/>

</xml_diff>